<commit_message>
Majopr update, revamped style, added uncertainty approach 1 and tornado sensitivity
</commit_message>
<xml_diff>
--- a/inst/extdata/example1-4pools.xlsx
+++ b/inst/extdata/example1-4pools.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gaelsola/Github-Collabs/mocaredd/inst/extdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gaelsola/code/mocaredd.dev2/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC83025B-AD59-1145-A8AE-F835164BAF7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B73094-9776-3343-87D7-BB9D86243189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1580" yWindow="760" windowWidth="28660" windowHeight="18880" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1220" yWindow="660" windowWidth="28180" windowHeight="18460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="11" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="129">
   <si>
     <t>trans_no</t>
   </si>
@@ -431,6 +431,9 @@
   </si>
   <si>
     <t>redd_activity</t>
+  </si>
+  <si>
+    <t>digits</t>
   </si>
 </sst>
 </file>
@@ -1032,7 +1035,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8C6B7CA-5E2C-284E-A17C-8E0897ACEFB0}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="8.5" bestFit="1" customWidth="1"/>
@@ -1045,7 +1048,7 @@
     <col min="9" max="9" width="13.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A1" s="25" t="s">
         <v>58</v>
       </c>
@@ -1079,8 +1082,11 @@
       <c r="K1" s="25" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="L1" s="25" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A2" t="b">
         <v>0</v>
       </c>
@@ -1113,6 +1119,9 @@
       </c>
       <c r="K2">
         <v>0.9</v>
+      </c>
+      <c r="L2">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>